<commit_message>
fix: add vite dependency
</commit_message>
<xml_diff>
--- a/inventario-ti/data/inventario_equipamentos_ti.xlsx
+++ b/inventario-ti/data/inventario_equipamentos_ti.xlsx
@@ -65,7 +65,7 @@
     <t>SN1234523489BR</t>
   </si>
   <si>
-    <t>Emprestado</t>
+    <t>Em manutenção</t>
   </si>
   <si>
     <t>Niteroi II</t>
@@ -956,9 +956,6 @@
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>20</v>
@@ -1146,6 +1143,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>